<commit_message>
Add professional README, Python scripts, and project assets
</commit_message>
<xml_diff>
--- a/1_Data_Sources/TreatmentDetails.xlsx
+++ b/1_Data_Sources/TreatmentDetails.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\12345\OneDrive\Desktop\biotech\sem 7\summer int, ppt\Diabetes_Treatment_Planner\1_Data_Sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8DE13CC8-0720-4CC1-BBB4-726C912ED99E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2C32170-749F-4599-BD08-9518B77067C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3216" yWindow="1344" windowWidth="17160" windowHeight="8976" xr2:uid="{7B3B6424-341C-4378-BB7C-B2F355C4F2AE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B3B6424-341C-4378-BB7C-B2F355C4F2AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Treatment_Details.xlsx" sheetId="1" r:id="rId1"/>
@@ -916,6 +916,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11FB1CC5-BBCB-4A78-BBA1-BADD859522EE}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.88671875" customWidth="1"/>
+    <col min="2" max="2" width="66.21875" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>